<commit_message>
Implement latest reports up to 7th Oct 2026
</commit_message>
<xml_diff>
--- a/data/Aug/Hàng trả từ ngày 24-31.xlsx
+++ b/data/Aug/Hàng trả từ ngày 24-31.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\Aug\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4EFAB77-78AD-4720-AB98-8F27FBE5415A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B47D6FA1-08AC-4C32-8678-B1B09603827D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -822,7 +822,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -855,6 +855,12 @@
       <i/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFC000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -905,7 +911,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -918,6 +924,9 @@
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1198,7 +1207,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R75"/>
+  <dimension ref="A1:S75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -2845,7 +2854,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5"/>
       <c r="B33" s="5" t="s">
         <v>16</v>
@@ -2894,8 +2903,10 @@
       <c r="Q33" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="R33" s="4"/>
+      <c r="S33" s="4"/>
+    </row>
+    <row r="34" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="2" t="s">
         <v>16</v>
@@ -2944,9 +2955,8 @@
       <c r="Q34" s="2">
         <v>1</v>
       </c>
-      <c r="R34" s="2"/>
-    </row>
-    <row r="35" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="2" t="s">
         <v>16</v>
@@ -2995,9 +3005,8 @@
       <c r="Q35" s="2">
         <v>1</v>
       </c>
-      <c r="R35" s="2"/>
-    </row>
-    <row r="36" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="2" t="s">
         <v>16</v>
@@ -3046,9 +3055,8 @@
       <c r="Q36" s="2">
         <v>1</v>
       </c>
-      <c r="R36" s="2"/>
-    </row>
-    <row r="37" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
       <c r="B37" s="2" t="s">
         <v>16</v>
@@ -3097,9 +3105,8 @@
       <c r="Q37" s="2">
         <v>1</v>
       </c>
-      <c r="R37" s="2"/>
-    </row>
-    <row r="38" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
       <c r="B38" s="2" t="s">
         <v>16</v>
@@ -3150,9 +3157,8 @@
       <c r="Q38" s="2">
         <v>1</v>
       </c>
-      <c r="R38" s="2"/>
-    </row>
-    <row r="39" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
       <c r="B39" s="2" t="s">
         <v>16</v>
@@ -3203,9 +3209,8 @@
       <c r="Q39" s="2">
         <v>1</v>
       </c>
-      <c r="R39" s="2"/>
-    </row>
-    <row r="40" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
       <c r="B40" s="2" t="s">
         <v>16</v>
@@ -3256,9 +3261,8 @@
       <c r="Q40" s="2">
         <v>1</v>
       </c>
-      <c r="R40" s="2"/>
-    </row>
-    <row r="41" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2"/>
       <c r="B41" s="2" t="s">
         <v>16</v>
@@ -3309,9 +3313,8 @@
       <c r="Q41" s="2">
         <v>1</v>
       </c>
-      <c r="R41" s="2"/>
-    </row>
-    <row r="42" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
       <c r="B42" s="2" t="s">
         <v>16</v>
@@ -3362,9 +3365,8 @@
       <c r="Q42" s="2">
         <v>1</v>
       </c>
-      <c r="R42" s="2"/>
-    </row>
-    <row r="43" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="1:19" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="5"/>
       <c r="B43" s="5" t="s">
         <v>16</v>
@@ -3415,9 +3417,10 @@
       <c r="Q43" s="5">
         <v>1</v>
       </c>
-      <c r="R43" s="5"/>
-    </row>
-    <row r="44" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="R43" s="4"/>
+      <c r="S43" s="4"/>
+    </row>
+    <row r="44" spans="1:19" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="5"/>
       <c r="B44" s="5" t="s">
         <v>16</v>
@@ -3468,9 +3471,10 @@
       <c r="Q44" s="5">
         <v>1</v>
       </c>
-      <c r="R44" s="5"/>
-    </row>
-    <row r="45" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="R44" s="4"/>
+      <c r="S44" s="4"/>
+    </row>
+    <row r="45" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2"/>
       <c r="B45" s="2" t="s">
         <v>16</v>
@@ -3521,9 +3525,8 @@
       <c r="Q45" s="2">
         <v>1</v>
       </c>
-      <c r="R45" s="2"/>
-    </row>
-    <row r="46" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="46" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2"/>
       <c r="B46" s="2" t="s">
         <v>16</v>
@@ -3574,9 +3577,8 @@
       <c r="Q46" s="2">
         <v>1</v>
       </c>
-      <c r="R46" s="2"/>
-    </row>
-    <row r="47" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="47" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2"/>
       <c r="B47" s="2" t="s">
         <v>16</v>
@@ -3627,9 +3629,8 @@
       <c r="Q47" s="2">
         <v>1</v>
       </c>
-      <c r="R47" s="2"/>
-    </row>
-    <row r="48" spans="1:18" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="48" spans="1:19" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="8"/>
       <c r="B48" s="8" t="s">
         <v>16</v>
@@ -3680,9 +3681,10 @@
       <c r="Q48" s="8">
         <v>1</v>
       </c>
-      <c r="R48" s="8"/>
-    </row>
-    <row r="49" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="R48" s="4"/>
+      <c r="S48" s="4"/>
+    </row>
+    <row r="49" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2"/>
       <c r="B49" s="2" t="s">
         <v>16</v>
@@ -3733,9 +3735,8 @@
       <c r="Q49" s="2">
         <v>1</v>
       </c>
-      <c r="R49" s="2"/>
-    </row>
-    <row r="50" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="50" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2"/>
       <c r="B50" s="2" t="s">
         <v>16</v>
@@ -3786,9 +3787,8 @@
       <c r="Q50" s="2">
         <v>1</v>
       </c>
-      <c r="R50" s="2"/>
-    </row>
-    <row r="51" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2"/>
       <c r="B51" s="2" t="s">
         <v>16</v>
@@ -3839,9 +3839,8 @@
       <c r="Q51" s="2">
         <v>1</v>
       </c>
-      <c r="R51" s="2"/>
-    </row>
-    <row r="52" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="52" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2"/>
       <c r="B52" s="2" t="s">
         <v>16</v>
@@ -3892,9 +3891,8 @@
       <c r="Q52" s="2">
         <v>1</v>
       </c>
-      <c r="R52" s="2"/>
-    </row>
-    <row r="53" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="53" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2"/>
       <c r="B53" s="2" t="s">
         <v>16</v>
@@ -3945,9 +3943,8 @@
       <c r="Q53" s="2">
         <v>1</v>
       </c>
-      <c r="R53" s="2"/>
-    </row>
-    <row r="54" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="54" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2"/>
       <c r="B54" s="2" t="s">
         <v>16</v>
@@ -3998,9 +3995,8 @@
       <c r="Q54" s="2">
         <v>1</v>
       </c>
-      <c r="R54" s="2"/>
-    </row>
-    <row r="55" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2"/>
       <c r="B55" s="2" t="s">
         <v>16</v>
@@ -4051,9 +4047,8 @@
       <c r="Q55" s="2">
         <v>1</v>
       </c>
-      <c r="R55" s="2"/>
-    </row>
-    <row r="56" spans="1:18" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="56" spans="1:19" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="8"/>
       <c r="B56" s="8" t="s">
         <v>16</v>
@@ -4104,9 +4099,10 @@
       <c r="Q56" s="8">
         <v>1</v>
       </c>
-      <c r="R56" s="8"/>
-    </row>
-    <row r="57" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="R56" s="4"/>
+      <c r="S56" s="4"/>
+    </row>
+    <row r="57" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2"/>
       <c r="B57" s="2" t="s">
         <v>16</v>
@@ -4157,9 +4153,8 @@
       <c r="Q57" s="2">
         <v>1</v>
       </c>
-      <c r="R57" s="2"/>
-    </row>
-    <row r="58" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2"/>
       <c r="B58" s="2" t="s">
         <v>16</v>
@@ -4210,9 +4205,8 @@
       <c r="Q58" s="2">
         <v>1</v>
       </c>
-      <c r="R58" s="2"/>
-    </row>
-    <row r="59" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="59" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2"/>
       <c r="B59" s="2" t="s">
         <v>16</v>
@@ -4263,9 +4257,8 @@
       <c r="Q59" s="2">
         <v>1</v>
       </c>
-      <c r="R59" s="3"/>
-    </row>
-    <row r="60" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="60" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2"/>
       <c r="B60" s="2" t="s">
         <v>16</v>
@@ -4316,9 +4309,8 @@
       <c r="Q60" s="2">
         <v>1</v>
       </c>
-      <c r="R60" s="2"/>
-    </row>
-    <row r="61" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="61" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2"/>
       <c r="B61" s="2" t="s">
         <v>16</v>
@@ -4369,9 +4361,8 @@
       <c r="Q61" s="2">
         <v>1</v>
       </c>
-      <c r="R61" s="2"/>
-    </row>
-    <row r="62" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="62" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2"/>
       <c r="B62" s="2" t="s">
         <v>16</v>
@@ -4423,103 +4414,103 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="2"/>
-      <c r="B63" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C63" s="2" t="s">
+    <row r="63" spans="1:19" s="14" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="12"/>
+      <c r="B63" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C63" s="12" t="s">
         <v>222</v>
       </c>
-      <c r="D63" s="2" t="s">
+      <c r="D63" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="E63" s="2" t="s">
+      <c r="E63" s="12" t="s">
         <v>223</v>
       </c>
-      <c r="F63" s="2" t="s">
+      <c r="F63" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="G63" s="3">
+      <c r="G63" s="13">
         <v>330</v>
       </c>
-      <c r="H63" s="3">
+      <c r="H63" s="13">
         <v>0</v>
       </c>
-      <c r="I63" s="3">
+      <c r="I63" s="13">
         <f t="shared" ref="I63" si="1">G63-H63</f>
         <v>330</v>
       </c>
-      <c r="J63" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K63" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L63" s="2" t="s">
+      <c r="J63" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K63" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="L63" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="M63" s="2" t="s">
+      <c r="M63" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="N63" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O63" s="2"/>
-      <c r="P63" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q63" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="2"/>
-      <c r="B64" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C64" s="2" t="s">
+      <c r="N63" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="O63" s="12"/>
+      <c r="P63" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q63" s="12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:19" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="12"/>
+      <c r="B64" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C64" s="12" t="s">
         <v>224</v>
       </c>
-      <c r="D64" s="2" t="s">
+      <c r="D64" s="12" t="s">
         <v>225</v>
       </c>
-      <c r="E64" s="2" t="s">
+      <c r="E64" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="F64" s="2" t="s">
+      <c r="F64" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="G64" s="3">
+      <c r="G64" s="13">
         <v>1650</v>
       </c>
-      <c r="H64" s="3">
+      <c r="H64" s="13">
         <v>0</v>
       </c>
-      <c r="I64" s="3">
+      <c r="I64" s="13">
         <f t="shared" ref="I64:I74" si="2">G64-H64</f>
         <v>1650</v>
       </c>
-      <c r="J64" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K64" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L64" s="2" t="s">
+      <c r="J64" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K64" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="L64" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="M64" s="2" t="s">
+      <c r="M64" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="N64" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O64" s="2"/>
-      <c r="P64" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q64" s="2">
+      <c r="N64" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="O64" s="12"/>
+      <c r="P64" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q64" s="12">
         <v>1</v>
       </c>
     </row>

</xml_diff>